<commit_message>
fix lai cccd, sua lai validate diem thi,bo validate cccd, them nut reset dashboard
</commit_message>
<xml_diff>
--- a/data/Uu tien xet tuyen.xlsx
+++ b/data/Uu tien xet tuyen.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/caothanh/Library/CloudStorage/GoogleDrive-caominhthanh99@gmail.com/My Drive/DayHoc/XDPMPL/2026/project_tuyensinh/"/>
     </mc:Choice>
@@ -22,7 +22,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5815" uniqueCount="672">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5542" uniqueCount="399">
   <si>
     <t>NV1</t>
   </si>
@@ -1246,832 +1246,12 @@
   </si>
   <si>
     <t>TS_22724</t>
-  </si>
-  <si>
-    <t>052307000028</t>
-  </si>
-  <si>
-    <t>038207000099</t>
-  </si>
-  <si>
-    <t>052307000027</t>
-  </si>
-  <si>
-    <t>034307000087</t>
-  </si>
-  <si>
-    <t>075307001426</t>
-  </si>
-  <si>
-    <t>079307007396</t>
-  </si>
-  <si>
-    <t>068307000305</t>
-  </si>
-  <si>
-    <t>068307000623</t>
-  </si>
-  <si>
-    <t>077307000213</t>
-  </si>
-  <si>
-    <t>075307000147</t>
-  </si>
-  <si>
-    <t>080207000259</t>
-  </si>
-  <si>
-    <t>079207001738</t>
-  </si>
-  <si>
-    <t>079307000197</t>
-  </si>
-  <si>
-    <t>079207005328</t>
-  </si>
-  <si>
-    <t>079207004767</t>
-  </si>
-  <si>
-    <t>054307000304</t>
-  </si>
-  <si>
-    <t>079307007958</t>
-  </si>
-  <si>
-    <t>075307001042</t>
-  </si>
-  <si>
-    <t>086307000147</t>
-  </si>
-  <si>
-    <t>031307000049</t>
-  </si>
-  <si>
-    <t>083307000540</t>
-  </si>
-  <si>
-    <t>079207005089</t>
-  </si>
-  <si>
-    <t>072205000002</t>
-  </si>
-  <si>
-    <t>077205000003</t>
-  </si>
-  <si>
-    <t>096207000064</t>
-  </si>
-  <si>
-    <t>079207002768</t>
-  </si>
-  <si>
-    <t>075307001490</t>
-  </si>
-  <si>
-    <t>060207000085</t>
-  </si>
-  <si>
-    <t>079307007228</t>
-  </si>
-  <si>
-    <t>091207000059</t>
-  </si>
-  <si>
-    <t>072307000005</t>
-  </si>
-  <si>
-    <t>091207000256</t>
-  </si>
-  <si>
-    <t>000307000160</t>
-  </si>
-  <si>
-    <t>079307008994</t>
-  </si>
-  <si>
-    <t>072307000177</t>
-  </si>
-  <si>
-    <t>079307007061</t>
-  </si>
-  <si>
-    <t>082207000390</t>
-  </si>
-  <si>
-    <t>082207000099</t>
-  </si>
-  <si>
-    <t>072207000247</t>
-  </si>
-  <si>
-    <t>079307007231</t>
-  </si>
-  <si>
-    <t>079207001695</t>
-  </si>
-  <si>
-    <t>079307004329</t>
-  </si>
-  <si>
-    <t>042207000091</t>
-  </si>
-  <si>
-    <t>070207000054</t>
-  </si>
-  <si>
-    <t>052207000211</t>
-  </si>
-  <si>
-    <t>075307001462</t>
-  </si>
-  <si>
-    <t>066307000307</t>
-  </si>
-  <si>
-    <t>079307007574</t>
-  </si>
-  <si>
-    <t>080206000005</t>
-  </si>
-  <si>
-    <t>066307000600</t>
-  </si>
-  <si>
-    <t>082307000479</t>
-  </si>
-  <si>
-    <t>089207000164</t>
-  </si>
-  <si>
-    <t>089307000215</t>
-  </si>
-  <si>
-    <t>095307000112</t>
-  </si>
-  <si>
-    <t>079307004491</t>
-  </si>
-  <si>
-    <t>079206000120</t>
-  </si>
-  <si>
-    <t>079207004907</t>
-  </si>
-  <si>
-    <t>074307000619</t>
-  </si>
-  <si>
-    <t>077306000009</t>
-  </si>
-  <si>
-    <t>082307000922</t>
-  </si>
-  <si>
-    <t>075207000086</t>
-  </si>
-  <si>
-    <t>096307000021</t>
-  </si>
-  <si>
-    <t>060207000352</t>
-  </si>
-  <si>
-    <t>075307000480</t>
-  </si>
-  <si>
-    <t>074307000414</t>
-  </si>
-  <si>
-    <t>079307006453</t>
-  </si>
-  <si>
-    <t>042307000182</t>
-  </si>
-  <si>
-    <t>091307000220</t>
-  </si>
-  <si>
-    <t>060307000215</t>
-  </si>
-  <si>
-    <t>079207002063</t>
-  </si>
-  <si>
-    <t>072207000023</t>
-  </si>
-  <si>
-    <t>083307000752</t>
-  </si>
-  <si>
-    <t>091207000126</t>
-  </si>
-  <si>
-    <t>038307000266</t>
-  </si>
-  <si>
-    <t>052307000052</t>
-  </si>
-  <si>
-    <t>075307000709</t>
-  </si>
-  <si>
-    <t>060207000357</t>
-  </si>
-  <si>
-    <t>080307000158</t>
-  </si>
-  <si>
-    <t>052307000461</t>
-  </si>
-  <si>
-    <t>094207000042</t>
-  </si>
-  <si>
-    <t>087207000225</t>
-  </si>
-  <si>
-    <t>091307000069</t>
-  </si>
-  <si>
-    <t>079207000972</t>
-  </si>
-  <si>
-    <t>036307000102</t>
-  </si>
-  <si>
-    <t>064207000193</t>
-  </si>
-  <si>
-    <t>045307000072</t>
-  </si>
-  <si>
-    <t>052307000706</t>
-  </si>
-  <si>
-    <t>066307000686</t>
-  </si>
-  <si>
-    <t>075307000826</t>
-  </si>
-  <si>
-    <t>051307000382</t>
-  </si>
-  <si>
-    <t>038307000137</t>
-  </si>
-  <si>
-    <t>091306000002</t>
-  </si>
-  <si>
-    <t>079307004985</t>
-  </si>
-  <si>
-    <t>079307007774</t>
-  </si>
-  <si>
-    <t>056207000065</t>
-  </si>
-  <si>
-    <t>074307000322</t>
-  </si>
-  <si>
-    <t>079307000341</t>
-  </si>
-  <si>
-    <t>052307000784</t>
-  </si>
-  <si>
-    <t>054307000213</t>
-  </si>
-  <si>
-    <t>067307000015</t>
-  </si>
-  <si>
-    <t>074206000015</t>
-  </si>
-  <si>
-    <t>094307000112</t>
-  </si>
-  <si>
-    <t>089207000111</t>
-  </si>
-  <si>
-    <t>072207000217</t>
-  </si>
-  <si>
-    <t>079307003353</t>
-  </si>
-  <si>
-    <t>070207000168</t>
-  </si>
-  <si>
-    <t>079205000018</t>
-  </si>
-  <si>
-    <t>079207002854</t>
-  </si>
-  <si>
-    <t>079307005075</t>
-  </si>
-  <si>
-    <t>074307000041</t>
-  </si>
-  <si>
-    <t>079305000033</t>
-  </si>
-  <si>
-    <t>079307004793</t>
-  </si>
-  <si>
-    <t>079307007961</t>
-  </si>
-  <si>
-    <t>079307003366</t>
-  </si>
-  <si>
-    <t>049207000106</t>
-  </si>
-  <si>
-    <t>079307000195</t>
-  </si>
-  <si>
-    <t>079207001749</t>
-  </si>
-  <si>
-    <t>001307000052</t>
-  </si>
-  <si>
-    <t>038307000475</t>
-  </si>
-  <si>
-    <t>079207005372</t>
-  </si>
-  <si>
-    <t>060307000797</t>
-  </si>
-  <si>
-    <t>066307000688</t>
-  </si>
-  <si>
-    <t>038307000229</t>
-  </si>
-  <si>
-    <t>079307008387</t>
-  </si>
-  <si>
-    <t>080307000249</t>
-  </si>
-  <si>
-    <t>079307001760</t>
-  </si>
-  <si>
-    <t>058307000227</t>
-  </si>
-  <si>
-    <t>079307004255</t>
-  </si>
-  <si>
-    <t>068207000159</t>
-  </si>
-  <si>
-    <t>040307000351</t>
-  </si>
-  <si>
-    <t>096307000371</t>
-  </si>
-  <si>
-    <t>095307000289</t>
-  </si>
-  <si>
-    <t>082307000426</t>
-  </si>
-  <si>
-    <t>075307001696</t>
-  </si>
-  <si>
-    <t>051207000031</t>
-  </si>
-  <si>
-    <t>089307000561</t>
-  </si>
-  <si>
-    <t>079307007223</t>
-  </si>
-  <si>
-    <t>079307006677</t>
-  </si>
-  <si>
-    <t>079207001030</t>
-  </si>
-  <si>
-    <t>079307001509</t>
-  </si>
-  <si>
-    <t>074307000756</t>
-  </si>
-  <si>
-    <t>079307005482</t>
-  </si>
-  <si>
-    <t>075307000749</t>
-  </si>
-  <si>
-    <t>089207000430</t>
-  </si>
-  <si>
-    <t>060207000169</t>
-  </si>
-  <si>
-    <t>056307000012</t>
-  </si>
-  <si>
-    <t>070307000661</t>
-  </si>
-  <si>
-    <t>079207000796</t>
-  </si>
-  <si>
-    <t>001307000002</t>
-  </si>
-  <si>
-    <t>079307002061</t>
-  </si>
-  <si>
-    <t>091307000171</t>
-  </si>
-  <si>
-    <t>095207000155</t>
-  </si>
-  <si>
-    <t>079307005042</t>
-  </si>
-  <si>
-    <t>086207000021</t>
-  </si>
-  <si>
-    <t>051207000136</t>
-  </si>
-  <si>
-    <t>054307000145</t>
-  </si>
-  <si>
-    <t>048207000005</t>
-  </si>
-  <si>
-    <t>079207000731</t>
-  </si>
-  <si>
-    <t>054206000001</t>
-  </si>
-  <si>
-    <t>080306000015</t>
-  </si>
-  <si>
-    <t>049307000192</t>
-  </si>
-  <si>
-    <t>066307000391</t>
-  </si>
-  <si>
-    <t>083307000259</t>
-  </si>
-  <si>
-    <t>068207000002</t>
-  </si>
-  <si>
-    <t>094207000077</t>
-  </si>
-  <si>
-    <t>060307000891</t>
-  </si>
-  <si>
-    <t>079307007498</t>
-  </si>
-  <si>
-    <t>079307007245</t>
-  </si>
-  <si>
-    <t>048307000037</t>
-  </si>
-  <si>
-    <t>075307000227</t>
-  </si>
-  <si>
-    <t>038207000062</t>
-  </si>
-  <si>
-    <t>066307000746</t>
-  </si>
-  <si>
-    <t>079307005551</t>
-  </si>
-  <si>
-    <t>079307006673</t>
-  </si>
-  <si>
-    <t>084307000113</t>
-  </si>
-  <si>
-    <t>070207000055</t>
-  </si>
-  <si>
-    <t>079207003113</t>
-  </si>
-  <si>
-    <t>068307000057</t>
-  </si>
-  <si>
-    <t>074307000300</t>
-  </si>
-  <si>
-    <t>079207002322</t>
-  </si>
-  <si>
-    <t>077307000388</t>
-  </si>
-  <si>
-    <t>079206000179</t>
-  </si>
-  <si>
-    <t>060307000271</t>
-  </si>
-  <si>
-    <t>079307005950</t>
-  </si>
-  <si>
-    <t>054307000314</t>
-  </si>
-  <si>
-    <t>070207000203</t>
-  </si>
-  <si>
-    <t>075207000507</t>
-  </si>
-  <si>
-    <t>094307000170</t>
-  </si>
-  <si>
-    <t>072307000269</t>
-  </si>
-  <si>
-    <t>066207000254</t>
-  </si>
-  <si>
-    <t>079306000034</t>
-  </si>
-  <si>
-    <t>060207000359</t>
-  </si>
-  <si>
-    <t>079307007486</t>
-  </si>
-  <si>
-    <t>080307000151</t>
-  </si>
-  <si>
-    <t>079207005027</t>
-  </si>
-  <si>
-    <t>082307000430</t>
-  </si>
-  <si>
-    <t>058307000339</t>
-  </si>
-  <si>
-    <t>056307000307</t>
-  </si>
-  <si>
-    <t>038307000338</t>
-  </si>
-  <si>
-    <t>079207003565</t>
-  </si>
-  <si>
-    <t>095207000043</t>
-  </si>
-  <si>
-    <t>089207000184</t>
-  </si>
-  <si>
-    <t>089307000515</t>
-  </si>
-  <si>
-    <t>062306000002</t>
-  </si>
-  <si>
-    <t>079307008194</t>
-  </si>
-  <si>
-    <t>062207000049</t>
-  </si>
-  <si>
-    <t>079207001617</t>
-  </si>
-  <si>
-    <t>079207001552</t>
-  </si>
-  <si>
-    <t>079303000006</t>
-  </si>
-  <si>
-    <t>052307000716</t>
-  </si>
-  <si>
-    <t>074307000001</t>
-  </si>
-  <si>
-    <t>079307004410</t>
-  </si>
-  <si>
-    <t>060307000287</t>
-  </si>
-  <si>
-    <t>079207003318</t>
-  </si>
-  <si>
-    <t>068207000063</t>
-  </si>
-  <si>
-    <t>060207000404</t>
-  </si>
-  <si>
-    <t>000307000191</t>
-  </si>
-  <si>
-    <t>072307000564</t>
-  </si>
-  <si>
-    <t>054206000004</t>
-  </si>
-  <si>
-    <t>066307000759</t>
-  </si>
-  <si>
-    <t>077307000325</t>
-  </si>
-  <si>
-    <t>079207001763</t>
-  </si>
-  <si>
-    <t>079307007300</t>
-  </si>
-  <si>
-    <t>051307000765</t>
-  </si>
-  <si>
-    <t>091207000237</t>
-  </si>
-  <si>
-    <t>068207000057</t>
-  </si>
-  <si>
-    <t>049207000087</t>
-  </si>
-  <si>
-    <t>072307000080</t>
-  </si>
-  <si>
-    <t>072307000276</t>
-  </si>
-  <si>
-    <t>056307000448</t>
-  </si>
-  <si>
-    <t>096307000012</t>
-  </si>
-  <si>
-    <t>094207000082</t>
-  </si>
-  <si>
-    <t>079207004459</t>
-  </si>
-  <si>
-    <t>079207003116</t>
-  </si>
-  <si>
-    <t>064307000196</t>
-  </si>
-  <si>
-    <t>075307000473</t>
-  </si>
-  <si>
-    <t>051201000001</t>
-  </si>
-  <si>
-    <t>079207003092</t>
-  </si>
-  <si>
-    <t>082307000387</t>
-  </si>
-  <si>
-    <t>038307000027</t>
-  </si>
-  <si>
-    <t>079207002575</t>
-  </si>
-  <si>
-    <t>079307006509</t>
-  </si>
-  <si>
-    <t>068307000502</t>
-  </si>
-  <si>
-    <t>075307001440</t>
-  </si>
-  <si>
-    <t>079207002612</t>
-  </si>
-  <si>
-    <t>079307008468</t>
-  </si>
-  <si>
-    <t>075307000970</t>
-  </si>
-  <si>
-    <t>091307000511</t>
-  </si>
-  <si>
-    <t>052207000375</t>
-  </si>
-  <si>
-    <t>038307000026</t>
-  </si>
-  <si>
-    <t>079307008748</t>
-  </si>
-  <si>
-    <t>095306000011</t>
-  </si>
-  <si>
-    <t>079307001213</t>
-  </si>
-  <si>
-    <t>019307000009</t>
-  </si>
-  <si>
-    <t>051207000040</t>
-  </si>
-  <si>
-    <t>079207002522</t>
-  </si>
-  <si>
-    <t>079307002816</t>
-  </si>
-  <si>
-    <t>079204000022</t>
-  </si>
-  <si>
-    <t>079207003188</t>
-  </si>
-  <si>
-    <t>089207000029</t>
-  </si>
-  <si>
-    <t>075207000573</t>
-  </si>
-  <si>
-    <t>034307000079</t>
-  </si>
-  <si>
-    <t>077307000745</t>
-  </si>
-  <si>
-    <t>079307005886</t>
-  </si>
-  <si>
-    <t>051307000098</t>
-  </si>
-  <si>
-    <t>054307000072</t>
-  </si>
-  <si>
-    <t>074307000049</t>
-  </si>
-  <si>
-    <t>080307000150</t>
-  </si>
-  <si>
-    <t>089307000232</t>
-  </si>
-  <si>
-    <t>079307003704</t>
-  </si>
-  <si>
-    <t>077207000243</t>
-  </si>
-  <si>
-    <t>077307000221</t>
-  </si>
-  <si>
-    <t>079307003874</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2594,13 +1774,13 @@
   <dimension ref="A1:I274"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="20" width="6.5"/>
-    <col min="2" max="2" customWidth="true" style="20" width="19.1640625"/>
-    <col min="3" max="4" customWidth="true" width="14.6640625"/>
-    <col min="5" max="5" customWidth="true" width="10.33203125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="16.83203125"/>
-    <col min="7" max="7" customWidth="true" style="1" width="13.5"/>
-    <col min="8" max="8" customWidth="true" style="1" width="20.5"/>
+    <col min="1" max="1" width="6.5" style="20" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" style="20" customWidth="1"/>
+    <col min="3" max="4" width="14.6640625" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5" style="1" customWidth="1"/>
+    <col min="8" max="8" width="20.5" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="32" x14ac:dyDescent="0.2">
@@ -2637,7 +1817,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>399</v>
+        <v>126</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>97</v>
@@ -2663,7 +1843,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>400</v>
+        <v>127</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>97</v>
@@ -2689,7 +1869,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>401</v>
+        <v>128</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>97</v>
@@ -2715,7 +1895,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>402</v>
+        <v>129</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>97</v>
@@ -2741,7 +1921,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>403</v>
+        <v>130</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>97</v>
@@ -2767,7 +1947,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>404</v>
+        <v>131</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>97</v>
@@ -2793,7 +1973,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>405</v>
+        <v>132</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>97</v>
@@ -2819,7 +1999,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>406</v>
+        <v>133</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>97</v>
@@ -2845,7 +2025,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>407</v>
+        <v>134</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>97</v>
@@ -2871,7 +2051,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>408</v>
+        <v>135</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>97</v>
@@ -2897,7 +2077,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>409</v>
+        <v>136</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>97</v>
@@ -2923,7 +2103,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>410</v>
+        <v>137</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>97</v>
@@ -2949,7 +2129,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>411</v>
+        <v>138</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>97</v>
@@ -2975,7 +2155,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>412</v>
+        <v>139</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>97</v>
@@ -3001,7 +2181,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>413</v>
+        <v>140</v>
       </c>
       <c r="C16" s="17" t="s">
         <v>97</v>
@@ -3027,7 +2207,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>414</v>
+        <v>141</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>98</v>
@@ -3053,7 +2233,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>415</v>
+        <v>142</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>98</v>
@@ -3079,7 +2259,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>416</v>
+        <v>143</v>
       </c>
       <c r="C19" s="8" t="s">
         <v>98</v>
@@ -3105,7 +2285,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>417</v>
+        <v>144</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>98</v>
@@ -3131,7 +2311,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>418</v>
+        <v>145</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>98</v>
@@ -3157,7 +2337,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>419</v>
+        <v>146</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>98</v>
@@ -3183,7 +2363,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>420</v>
+        <v>147</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>98</v>
@@ -3209,7 +2389,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>421</v>
+        <v>148</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>98</v>
@@ -3235,7 +2415,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>422</v>
+        <v>149</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>98</v>
@@ -3261,7 +2441,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>423</v>
+        <v>150</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>98</v>
@@ -3287,7 +2467,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>424</v>
+        <v>151</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>98</v>
@@ -3313,7 +2493,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>425</v>
+        <v>152</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>98</v>
@@ -3339,7 +2519,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>426</v>
+        <v>153</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>98</v>
@@ -3365,7 +2545,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>427</v>
+        <v>154</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>98</v>
@@ -3391,7 +2571,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>428</v>
+        <v>155</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>98</v>
@@ -3417,7 +2597,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>429</v>
+        <v>156</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>98</v>
@@ -3443,7 +2623,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>430</v>
+        <v>157</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>98</v>
@@ -3469,7 +2649,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>431</v>
+        <v>158</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>98</v>
@@ -3495,7 +2675,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>432</v>
+        <v>159</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>98</v>
@@ -3521,7 +2701,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>433</v>
+        <v>160</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>98</v>
@@ -3547,7 +2727,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>434</v>
+        <v>161</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>98</v>
@@ -3573,7 +2753,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>435</v>
+        <v>162</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>98</v>
@@ -3599,7 +2779,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>436</v>
+        <v>163</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>98</v>
@@ -3625,7 +2805,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>437</v>
+        <v>164</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>98</v>
@@ -3651,7 +2831,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>438</v>
+        <v>165</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>98</v>
@@ -3677,7 +2857,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>439</v>
+        <v>166</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>98</v>
@@ -3703,7 +2883,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>440</v>
+        <v>167</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>98</v>
@@ -3729,7 +2909,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>441</v>
+        <v>168</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>98</v>
@@ -3755,7 +2935,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>442</v>
+        <v>169</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>98</v>
@@ -3781,7 +2961,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>443</v>
+        <v>170</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>98</v>
@@ -3807,7 +2987,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>444</v>
+        <v>171</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>98</v>
@@ -3833,7 +3013,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>445</v>
+        <v>172</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>98</v>
@@ -3859,7 +3039,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="20" t="s">
-        <v>446</v>
+        <v>173</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>98</v>
@@ -3885,7 +3065,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>447</v>
+        <v>174</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>98</v>
@@ -3911,7 +3091,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>448</v>
+        <v>175</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>98</v>
@@ -3937,7 +3117,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>449</v>
+        <v>176</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>98</v>
@@ -3963,7 +3143,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="20" t="s">
-        <v>450</v>
+        <v>177</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>98</v>
@@ -3989,7 +3169,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>451</v>
+        <v>178</v>
       </c>
       <c r="C54" s="5" t="s">
         <v>98</v>
@@ -4015,7 +3195,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>452</v>
+        <v>179</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>98</v>
@@ -4041,7 +3221,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>453</v>
+        <v>180</v>
       </c>
       <c r="C56" s="5" t="s">
         <v>98</v>
@@ -4067,7 +3247,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="20" t="s">
-        <v>454</v>
+        <v>181</v>
       </c>
       <c r="C57" s="5" t="s">
         <v>98</v>
@@ -4093,7 +3273,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="20" t="s">
-        <v>455</v>
+        <v>182</v>
       </c>
       <c r="C58" s="8" t="s">
         <v>98</v>
@@ -4119,7 +3299,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="20" t="s">
-        <v>456</v>
+        <v>183</v>
       </c>
       <c r="C59" s="5" t="s">
         <v>98</v>
@@ -4145,7 +3325,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>457</v>
+        <v>184</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>98</v>
@@ -4171,7 +3351,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>458</v>
+        <v>185</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>98</v>
@@ -4197,7 +3377,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="20" t="s">
-        <v>459</v>
+        <v>186</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>98</v>
@@ -4223,7 +3403,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="20" t="s">
-        <v>460</v>
+        <v>187</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>98</v>
@@ -4249,7 +3429,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="20" t="s">
-        <v>461</v>
+        <v>188</v>
       </c>
       <c r="C64" s="5" t="s">
         <v>98</v>
@@ -4275,7 +3455,7 @@
         <v>64</v>
       </c>
       <c r="B65" s="20" t="s">
-        <v>462</v>
+        <v>189</v>
       </c>
       <c r="C65" s="5" t="s">
         <v>98</v>
@@ -4301,7 +3481,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>463</v>
+        <v>190</v>
       </c>
       <c r="C66" s="5" t="s">
         <v>98</v>
@@ -4327,7 +3507,7 @@
         <v>66</v>
       </c>
       <c r="B67" s="20" t="s">
-        <v>464</v>
+        <v>191</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>98</v>
@@ -4353,7 +3533,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="20" t="s">
-        <v>465</v>
+        <v>192</v>
       </c>
       <c r="C68" s="5" t="s">
         <v>98</v>
@@ -4379,7 +3559,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="20" t="s">
-        <v>466</v>
+        <v>193</v>
       </c>
       <c r="C69" s="5" t="s">
         <v>98</v>
@@ -4405,7 +3585,7 @@
         <v>69</v>
       </c>
       <c r="B70" s="20" t="s">
-        <v>467</v>
+        <v>194</v>
       </c>
       <c r="C70" s="5" t="s">
         <v>98</v>
@@ -4431,7 +3611,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="20" t="s">
-        <v>468</v>
+        <v>195</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>98</v>
@@ -4457,7 +3637,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="20" t="s">
-        <v>469</v>
+        <v>196</v>
       </c>
       <c r="C72" s="5" t="s">
         <v>98</v>
@@ -4483,7 +3663,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="20" t="s">
-        <v>470</v>
+        <v>197</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>98</v>
@@ -4509,7 +3689,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="20" t="s">
-        <v>471</v>
+        <v>198</v>
       </c>
       <c r="C74" s="5" t="s">
         <v>98</v>
@@ -4535,7 +3715,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="20" t="s">
-        <v>472</v>
+        <v>199</v>
       </c>
       <c r="C75" s="5" t="s">
         <v>98</v>
@@ -4561,7 +3741,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="20" t="s">
-        <v>473</v>
+        <v>200</v>
       </c>
       <c r="C76" s="8" t="s">
         <v>98</v>
@@ -4587,7 +3767,7 @@
         <v>76</v>
       </c>
       <c r="B77" s="20" t="s">
-        <v>474</v>
+        <v>201</v>
       </c>
       <c r="C77" s="8" t="s">
         <v>98</v>
@@ -4613,7 +3793,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="20" t="s">
-        <v>475</v>
+        <v>202</v>
       </c>
       <c r="C78" s="8" t="s">
         <v>98</v>
@@ -4639,7 +3819,7 @@
         <v>78</v>
       </c>
       <c r="B79" s="20" t="s">
-        <v>476</v>
+        <v>203</v>
       </c>
       <c r="C79" s="5" t="s">
         <v>98</v>
@@ -4665,7 +3845,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="20" t="s">
-        <v>477</v>
+        <v>204</v>
       </c>
       <c r="C80" s="8" t="s">
         <v>98</v>
@@ -4691,7 +3871,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="20" t="s">
-        <v>478</v>
+        <v>205</v>
       </c>
       <c r="C81" s="5" t="s">
         <v>98</v>
@@ -4717,7 +3897,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="20" t="s">
-        <v>479</v>
+        <v>206</v>
       </c>
       <c r="C82" s="5" t="s">
         <v>98</v>
@@ -4743,7 +3923,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="20" t="s">
-        <v>480</v>
+        <v>207</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>98</v>
@@ -4769,7 +3949,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="20" t="s">
-        <v>481</v>
+        <v>208</v>
       </c>
       <c r="C84" s="8" t="s">
         <v>98</v>
@@ -4795,7 +3975,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="20" t="s">
-        <v>482</v>
+        <v>209</v>
       </c>
       <c r="C85" s="5" t="s">
         <v>98</v>
@@ -4821,7 +4001,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="20" t="s">
-        <v>483</v>
+        <v>210</v>
       </c>
       <c r="C86" s="5" t="s">
         <v>98</v>
@@ -4847,7 +4027,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="20" t="s">
-        <v>484</v>
+        <v>211</v>
       </c>
       <c r="C87" s="5" t="s">
         <v>98</v>
@@ -4873,7 +4053,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="20" t="s">
-        <v>485</v>
+        <v>212</v>
       </c>
       <c r="C88" s="5" t="s">
         <v>98</v>
@@ -4899,7 +4079,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="20" t="s">
-        <v>486</v>
+        <v>213</v>
       </c>
       <c r="C89" s="8" t="s">
         <v>98</v>
@@ -4925,7 +4105,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="20" t="s">
-        <v>487</v>
+        <v>214</v>
       </c>
       <c r="C90" s="5" t="s">
         <v>98</v>
@@ -4951,7 +4131,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="20" t="s">
-        <v>488</v>
+        <v>215</v>
       </c>
       <c r="C91" s="8" t="s">
         <v>98</v>
@@ -4977,7 +4157,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="20" t="s">
-        <v>489</v>
+        <v>216</v>
       </c>
       <c r="C92" s="8" t="s">
         <v>98</v>
@@ -5003,7 +4183,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="20" t="s">
-        <v>490</v>
+        <v>217</v>
       </c>
       <c r="C93" s="5" t="s">
         <v>98</v>
@@ -5029,7 +4209,7 @@
         <v>93</v>
       </c>
       <c r="B94" s="20" t="s">
-        <v>491</v>
+        <v>218</v>
       </c>
       <c r="C94" s="5" t="s">
         <v>98</v>
@@ -5055,7 +4235,7 @@
         <v>94</v>
       </c>
       <c r="B95" s="20" t="s">
-        <v>492</v>
+        <v>219</v>
       </c>
       <c r="C95" s="8" t="s">
         <v>98</v>
@@ -5081,7 +4261,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="20" t="s">
-        <v>493</v>
+        <v>220</v>
       </c>
       <c r="C96" s="8" t="s">
         <v>98</v>
@@ -5107,7 +4287,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="20" t="s">
-        <v>494</v>
+        <v>221</v>
       </c>
       <c r="C97" s="8" t="s">
         <v>98</v>
@@ -5133,7 +4313,7 @@
         <v>97</v>
       </c>
       <c r="B98" s="20" t="s">
-        <v>495</v>
+        <v>222</v>
       </c>
       <c r="C98" s="8" t="s">
         <v>98</v>
@@ -5159,7 +4339,7 @@
         <v>98</v>
       </c>
       <c r="B99" s="20" t="s">
-        <v>496</v>
+        <v>223</v>
       </c>
       <c r="C99" s="5" t="s">
         <v>98</v>
@@ -5185,7 +4365,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="20" t="s">
-        <v>497</v>
+        <v>224</v>
       </c>
       <c r="C100" s="8" t="s">
         <v>98</v>
@@ -5211,7 +4391,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="20" t="s">
-        <v>498</v>
+        <v>225</v>
       </c>
       <c r="C101" s="5" t="s">
         <v>98</v>
@@ -5237,7 +4417,7 @@
         <v>101</v>
       </c>
       <c r="B102" s="20" t="s">
-        <v>499</v>
+        <v>226</v>
       </c>
       <c r="C102" s="8" t="s">
         <v>98</v>
@@ -5263,7 +4443,7 @@
         <v>102</v>
       </c>
       <c r="B103" s="20" t="s">
-        <v>500</v>
+        <v>227</v>
       </c>
       <c r="C103" s="5" t="s">
         <v>98</v>
@@ -5289,7 +4469,7 @@
         <v>103</v>
       </c>
       <c r="B104" s="20" t="s">
-        <v>501</v>
+        <v>228</v>
       </c>
       <c r="C104" s="5" t="s">
         <v>98</v>
@@ -5315,7 +4495,7 @@
         <v>104</v>
       </c>
       <c r="B105" s="20" t="s">
-        <v>502</v>
+        <v>229</v>
       </c>
       <c r="C105" s="5" t="s">
         <v>98</v>
@@ -5341,7 +4521,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="20" t="s">
-        <v>503</v>
+        <v>230</v>
       </c>
       <c r="C106" s="8" t="s">
         <v>98</v>
@@ -5367,7 +4547,7 @@
         <v>106</v>
       </c>
       <c r="B107" s="20" t="s">
-        <v>504</v>
+        <v>231</v>
       </c>
       <c r="C107" s="5" t="s">
         <v>98</v>
@@ -5393,7 +4573,7 @@
         <v>107</v>
       </c>
       <c r="B108" s="20" t="s">
-        <v>505</v>
+        <v>232</v>
       </c>
       <c r="C108" s="8" t="s">
         <v>98</v>
@@ -5419,7 +4599,7 @@
         <v>108</v>
       </c>
       <c r="B109" s="20" t="s">
-        <v>506</v>
+        <v>233</v>
       </c>
       <c r="C109" s="5" t="s">
         <v>98</v>
@@ -5445,7 +4625,7 @@
         <v>109</v>
       </c>
       <c r="B110" s="20" t="s">
-        <v>507</v>
+        <v>234</v>
       </c>
       <c r="C110" s="5" t="s">
         <v>98</v>
@@ -5471,7 +4651,7 @@
         <v>110</v>
       </c>
       <c r="B111" s="20" t="s">
-        <v>508</v>
+        <v>235</v>
       </c>
       <c r="C111" s="8" t="s">
         <v>98</v>
@@ -5497,7 +4677,7 @@
         <v>111</v>
       </c>
       <c r="B112" s="20" t="s">
-        <v>509</v>
+        <v>236</v>
       </c>
       <c r="C112" s="5" t="s">
         <v>98</v>
@@ -5523,7 +4703,7 @@
         <v>112</v>
       </c>
       <c r="B113" s="20" t="s">
-        <v>510</v>
+        <v>237</v>
       </c>
       <c r="C113" s="5" t="s">
         <v>98</v>
@@ -5549,7 +4729,7 @@
         <v>113</v>
       </c>
       <c r="B114" s="20" t="s">
-        <v>511</v>
+        <v>238</v>
       </c>
       <c r="C114" s="5" t="s">
         <v>98</v>
@@ -5575,7 +4755,7 @@
         <v>114</v>
       </c>
       <c r="B115" s="20" t="s">
-        <v>512</v>
+        <v>239</v>
       </c>
       <c r="C115" s="5" t="s">
         <v>98</v>
@@ -5601,7 +4781,7 @@
         <v>115</v>
       </c>
       <c r="B116" s="20" t="s">
-        <v>513</v>
+        <v>240</v>
       </c>
       <c r="C116" s="8" t="s">
         <v>98</v>
@@ -5627,7 +4807,7 @@
         <v>116</v>
       </c>
       <c r="B117" s="20" t="s">
-        <v>514</v>
+        <v>241</v>
       </c>
       <c r="C117" s="5" t="s">
         <v>98</v>
@@ -5653,7 +4833,7 @@
         <v>117</v>
       </c>
       <c r="B118" s="20" t="s">
-        <v>515</v>
+        <v>242</v>
       </c>
       <c r="C118" s="8" t="s">
         <v>98</v>
@@ -5679,7 +4859,7 @@
         <v>118</v>
       </c>
       <c r="B119" s="20" t="s">
-        <v>516</v>
+        <v>243</v>
       </c>
       <c r="C119" s="5" t="s">
         <v>98</v>
@@ -5705,7 +4885,7 @@
         <v>119</v>
       </c>
       <c r="B120" s="20" t="s">
-        <v>517</v>
+        <v>244</v>
       </c>
       <c r="C120" s="8" t="s">
         <v>98</v>
@@ -5731,7 +4911,7 @@
         <v>120</v>
       </c>
       <c r="B121" s="20" t="s">
-        <v>518</v>
+        <v>245</v>
       </c>
       <c r="C121" s="8" t="s">
         <v>98</v>
@@ -5757,7 +4937,7 @@
         <v>121</v>
       </c>
       <c r="B122" s="20" t="s">
-        <v>519</v>
+        <v>246</v>
       </c>
       <c r="C122" s="5" t="s">
         <v>98</v>
@@ -5783,7 +4963,7 @@
         <v>122</v>
       </c>
       <c r="B123" s="20" t="s">
-        <v>520</v>
+        <v>247</v>
       </c>
       <c r="C123" s="5" t="s">
         <v>98</v>
@@ -5809,7 +4989,7 @@
         <v>123</v>
       </c>
       <c r="B124" s="20" t="s">
-        <v>521</v>
+        <v>248</v>
       </c>
       <c r="C124" s="5" t="s">
         <v>98</v>
@@ -5835,7 +5015,7 @@
         <v>124</v>
       </c>
       <c r="B125" s="20" t="s">
-        <v>522</v>
+        <v>249</v>
       </c>
       <c r="C125" s="8" t="s">
         <v>98</v>
@@ -5861,7 +5041,7 @@
         <v>125</v>
       </c>
       <c r="B126" s="20" t="s">
-        <v>523</v>
+        <v>250</v>
       </c>
       <c r="C126" s="5" t="s">
         <v>98</v>
@@ -5887,7 +5067,7 @@
         <v>126</v>
       </c>
       <c r="B127" s="20" t="s">
-        <v>524</v>
+        <v>251</v>
       </c>
       <c r="C127" s="5" t="s">
         <v>98</v>
@@ -5913,7 +5093,7 @@
         <v>127</v>
       </c>
       <c r="B128" s="20" t="s">
-        <v>525</v>
+        <v>252</v>
       </c>
       <c r="C128" s="5" t="s">
         <v>98</v>
@@ -5939,7 +5119,7 @@
         <v>128</v>
       </c>
       <c r="B129" s="20" t="s">
-        <v>526</v>
+        <v>253</v>
       </c>
       <c r="C129" s="5" t="s">
         <v>98</v>
@@ -5965,7 +5145,7 @@
         <v>129</v>
       </c>
       <c r="B130" s="20" t="s">
-        <v>527</v>
+        <v>254</v>
       </c>
       <c r="C130" s="8" t="s">
         <v>98</v>
@@ -5991,7 +5171,7 @@
         <v>130</v>
       </c>
       <c r="B131" s="20" t="s">
-        <v>528</v>
+        <v>255</v>
       </c>
       <c r="C131" s="5" t="s">
         <v>98</v>
@@ -6017,7 +5197,7 @@
         <v>131</v>
       </c>
       <c r="B132" s="20" t="s">
-        <v>529</v>
+        <v>256</v>
       </c>
       <c r="C132" s="8" t="s">
         <v>98</v>
@@ -6043,7 +5223,7 @@
         <v>132</v>
       </c>
       <c r="B133" s="20" t="s">
-        <v>530</v>
+        <v>257</v>
       </c>
       <c r="C133" s="5" t="s">
         <v>98</v>
@@ -6069,7 +5249,7 @@
         <v>133</v>
       </c>
       <c r="B134" s="20" t="s">
-        <v>531</v>
+        <v>258</v>
       </c>
       <c r="C134" s="5" t="s">
         <v>98</v>
@@ -6095,7 +5275,7 @@
         <v>134</v>
       </c>
       <c r="B135" s="20" t="s">
-        <v>532</v>
+        <v>259</v>
       </c>
       <c r="C135" s="5" t="s">
         <v>98</v>
@@ -6121,7 +5301,7 @@
         <v>135</v>
       </c>
       <c r="B136" s="20" t="s">
-        <v>533</v>
+        <v>260</v>
       </c>
       <c r="C136" s="5" t="s">
         <v>98</v>
@@ -6147,7 +5327,7 @@
         <v>136</v>
       </c>
       <c r="B137" s="20" t="s">
-        <v>534</v>
+        <v>261</v>
       </c>
       <c r="C137" s="8" t="s">
         <v>98</v>
@@ -6173,7 +5353,7 @@
         <v>137</v>
       </c>
       <c r="B138" s="20" t="s">
-        <v>535</v>
+        <v>262</v>
       </c>
       <c r="C138" s="8" t="s">
         <v>98</v>
@@ -6199,7 +5379,7 @@
         <v>138</v>
       </c>
       <c r="B139" s="20" t="s">
-        <v>536</v>
+        <v>263</v>
       </c>
       <c r="C139" s="5" t="s">
         <v>98</v>
@@ -6225,7 +5405,7 @@
         <v>139</v>
       </c>
       <c r="B140" s="20" t="s">
-        <v>537</v>
+        <v>264</v>
       </c>
       <c r="C140" s="8" t="s">
         <v>98</v>
@@ -6251,7 +5431,7 @@
         <v>140</v>
       </c>
       <c r="B141" s="20" t="s">
-        <v>538</v>
+        <v>265</v>
       </c>
       <c r="C141" s="5" t="s">
         <v>98</v>
@@ -6277,7 +5457,7 @@
         <v>141</v>
       </c>
       <c r="B142" s="20" t="s">
-        <v>539</v>
+        <v>266</v>
       </c>
       <c r="C142" s="5" t="s">
         <v>98</v>
@@ -6303,7 +5483,7 @@
         <v>142</v>
       </c>
       <c r="B143" s="20" t="s">
-        <v>540</v>
+        <v>267</v>
       </c>
       <c r="C143" s="5" t="s">
         <v>98</v>
@@ -6329,7 +5509,7 @@
         <v>143</v>
       </c>
       <c r="B144" s="20" t="s">
-        <v>541</v>
+        <v>268</v>
       </c>
       <c r="C144" s="5" t="s">
         <v>98</v>
@@ -6355,7 +5535,7 @@
         <v>144</v>
       </c>
       <c r="B145" s="20" t="s">
-        <v>542</v>
+        <v>269</v>
       </c>
       <c r="C145" s="5" t="s">
         <v>98</v>
@@ -6381,7 +5561,7 @@
         <v>145</v>
       </c>
       <c r="B146" s="20" t="s">
-        <v>543</v>
+        <v>270</v>
       </c>
       <c r="C146" s="8" t="s">
         <v>98</v>
@@ -6407,7 +5587,7 @@
         <v>146</v>
       </c>
       <c r="B147" s="20" t="s">
-        <v>544</v>
+        <v>271</v>
       </c>
       <c r="C147" s="8" t="s">
         <v>98</v>
@@ -6433,7 +5613,7 @@
         <v>147</v>
       </c>
       <c r="B148" s="20" t="s">
-        <v>545</v>
+        <v>272</v>
       </c>
       <c r="C148" s="5" t="s">
         <v>98</v>
@@ -6459,7 +5639,7 @@
         <v>148</v>
       </c>
       <c r="B149" s="20" t="s">
-        <v>546</v>
+        <v>273</v>
       </c>
       <c r="C149" s="8" t="s">
         <v>98</v>
@@ -6485,7 +5665,7 @@
         <v>149</v>
       </c>
       <c r="B150" s="20" t="s">
-        <v>547</v>
+        <v>274</v>
       </c>
       <c r="C150" s="5" t="s">
         <v>98</v>
@@ -6511,7 +5691,7 @@
         <v>150</v>
       </c>
       <c r="B151" s="20" t="s">
-        <v>548</v>
+        <v>275</v>
       </c>
       <c r="C151" s="8" t="s">
         <v>98</v>
@@ -6537,7 +5717,7 @@
         <v>151</v>
       </c>
       <c r="B152" s="20" t="s">
-        <v>549</v>
+        <v>276</v>
       </c>
       <c r="C152" s="5" t="s">
         <v>98</v>
@@ -6563,7 +5743,7 @@
         <v>152</v>
       </c>
       <c r="B153" s="20" t="s">
-        <v>550</v>
+        <v>277</v>
       </c>
       <c r="C153" s="5" t="s">
         <v>98</v>
@@ -6589,7 +5769,7 @@
         <v>153</v>
       </c>
       <c r="B154" s="20" t="s">
-        <v>551</v>
+        <v>278</v>
       </c>
       <c r="C154" s="5" t="s">
         <v>98</v>
@@ -6615,7 +5795,7 @@
         <v>154</v>
       </c>
       <c r="B155" s="20" t="s">
-        <v>552</v>
+        <v>279</v>
       </c>
       <c r="C155" s="8" t="s">
         <v>98</v>
@@ -6641,7 +5821,7 @@
         <v>155</v>
       </c>
       <c r="B156" s="20" t="s">
-        <v>553</v>
+        <v>280</v>
       </c>
       <c r="C156" s="5" t="s">
         <v>98</v>
@@ -6667,7 +5847,7 @@
         <v>156</v>
       </c>
       <c r="B157" s="20" t="s">
-        <v>554</v>
+        <v>281</v>
       </c>
       <c r="C157" s="8" t="s">
         <v>98</v>
@@ -6693,7 +5873,7 @@
         <v>157</v>
       </c>
       <c r="B158" s="20" t="s">
-        <v>555</v>
+        <v>282</v>
       </c>
       <c r="C158" s="5" t="s">
         <v>98</v>
@@ -6719,7 +5899,7 @@
         <v>158</v>
       </c>
       <c r="B159" s="20" t="s">
-        <v>556</v>
+        <v>283</v>
       </c>
       <c r="C159" s="8" t="s">
         <v>98</v>
@@ -6745,7 +5925,7 @@
         <v>159</v>
       </c>
       <c r="B160" s="20" t="s">
-        <v>557</v>
+        <v>284</v>
       </c>
       <c r="C160" s="5" t="s">
         <v>98</v>
@@ -6771,7 +5951,7 @@
         <v>160</v>
       </c>
       <c r="B161" s="20" t="s">
-        <v>558</v>
+        <v>285</v>
       </c>
       <c r="C161" s="5" t="s">
         <v>98</v>
@@ -6797,7 +5977,7 @@
         <v>161</v>
       </c>
       <c r="B162" s="20" t="s">
-        <v>559</v>
+        <v>286</v>
       </c>
       <c r="C162" s="5" t="s">
         <v>98</v>
@@ -6823,7 +6003,7 @@
         <v>162</v>
       </c>
       <c r="B163" s="20" t="s">
-        <v>560</v>
+        <v>287</v>
       </c>
       <c r="C163" s="5" t="s">
         <v>98</v>
@@ -6849,7 +6029,7 @@
         <v>163</v>
       </c>
       <c r="B164" s="20" t="s">
-        <v>561</v>
+        <v>288</v>
       </c>
       <c r="C164" s="8" t="s">
         <v>98</v>
@@ -6875,7 +6055,7 @@
         <v>164</v>
       </c>
       <c r="B165" s="20" t="s">
-        <v>562</v>
+        <v>289</v>
       </c>
       <c r="C165" s="5" t="s">
         <v>98</v>
@@ -6901,7 +6081,7 @@
         <v>165</v>
       </c>
       <c r="B166" s="20" t="s">
-        <v>563</v>
+        <v>290</v>
       </c>
       <c r="C166" s="5" t="s">
         <v>98</v>
@@ -6927,7 +6107,7 @@
         <v>166</v>
       </c>
       <c r="B167" s="20" t="s">
-        <v>564</v>
+        <v>291</v>
       </c>
       <c r="C167" s="5" t="s">
         <v>98</v>
@@ -6953,7 +6133,7 @@
         <v>167</v>
       </c>
       <c r="B168" s="20" t="s">
-        <v>565</v>
+        <v>292</v>
       </c>
       <c r="C168" s="8" t="s">
         <v>98</v>
@@ -6979,7 +6159,7 @@
         <v>168</v>
       </c>
       <c r="B169" s="20" t="s">
-        <v>566</v>
+        <v>293</v>
       </c>
       <c r="C169" s="8" t="s">
         <v>98</v>
@@ -7005,7 +6185,7 @@
         <v>169</v>
       </c>
       <c r="B170" s="20" t="s">
-        <v>567</v>
+        <v>294</v>
       </c>
       <c r="C170" s="8" t="s">
         <v>98</v>
@@ -7031,7 +6211,7 @@
         <v>170</v>
       </c>
       <c r="B171" s="20" t="s">
-        <v>568</v>
+        <v>295</v>
       </c>
       <c r="C171" s="8" t="s">
         <v>98</v>
@@ -7057,7 +6237,7 @@
         <v>171</v>
       </c>
       <c r="B172" s="20" t="s">
-        <v>569</v>
+        <v>296</v>
       </c>
       <c r="C172" s="5" t="s">
         <v>98</v>
@@ -7083,7 +6263,7 @@
         <v>172</v>
       </c>
       <c r="B173" s="20" t="s">
-        <v>570</v>
+        <v>297</v>
       </c>
       <c r="C173" s="5" t="s">
         <v>98</v>
@@ -7109,7 +6289,7 @@
         <v>173</v>
       </c>
       <c r="B174" s="20" t="s">
-        <v>571</v>
+        <v>298</v>
       </c>
       <c r="C174" s="8" t="s">
         <v>98</v>
@@ -7135,7 +6315,7 @@
         <v>174</v>
       </c>
       <c r="B175" s="20" t="s">
-        <v>572</v>
+        <v>299</v>
       </c>
       <c r="C175" s="5" t="s">
         <v>98</v>
@@ -7161,7 +6341,7 @@
         <v>175</v>
       </c>
       <c r="B176" s="20" t="s">
-        <v>573</v>
+        <v>300</v>
       </c>
       <c r="C176" s="5" t="s">
         <v>98</v>
@@ -7187,7 +6367,7 @@
         <v>176</v>
       </c>
       <c r="B177" s="20" t="s">
-        <v>574</v>
+        <v>301</v>
       </c>
       <c r="C177" s="8" t="s">
         <v>98</v>
@@ -7213,7 +6393,7 @@
         <v>177</v>
       </c>
       <c r="B178" s="20" t="s">
-        <v>575</v>
+        <v>302</v>
       </c>
       <c r="C178" s="5" t="s">
         <v>98</v>
@@ -7239,7 +6419,7 @@
         <v>178</v>
       </c>
       <c r="B179" s="20" t="s">
-        <v>576</v>
+        <v>303</v>
       </c>
       <c r="C179" s="8" t="s">
         <v>98</v>
@@ -7265,7 +6445,7 @@
         <v>179</v>
       </c>
       <c r="B180" s="20" t="s">
-        <v>577</v>
+        <v>304</v>
       </c>
       <c r="C180" s="8" t="s">
         <v>98</v>
@@ -7291,7 +6471,7 @@
         <v>180</v>
       </c>
       <c r="B181" s="20" t="s">
-        <v>578</v>
+        <v>305</v>
       </c>
       <c r="C181" s="8" t="s">
         <v>98</v>
@@ -7317,7 +6497,7 @@
         <v>181</v>
       </c>
       <c r="B182" s="20" t="s">
-        <v>579</v>
+        <v>306</v>
       </c>
       <c r="C182" s="5" t="s">
         <v>98</v>
@@ -7343,7 +6523,7 @@
         <v>182</v>
       </c>
       <c r="B183" s="20" t="s">
-        <v>580</v>
+        <v>307</v>
       </c>
       <c r="C183" s="8" t="s">
         <v>98</v>
@@ -7369,7 +6549,7 @@
         <v>183</v>
       </c>
       <c r="B184" s="20" t="s">
-        <v>581</v>
+        <v>308</v>
       </c>
       <c r="C184" s="8" t="s">
         <v>98</v>
@@ -7395,7 +6575,7 @@
         <v>184</v>
       </c>
       <c r="B185" s="20" t="s">
-        <v>582</v>
+        <v>309</v>
       </c>
       <c r="C185" s="8" t="s">
         <v>98</v>
@@ -7421,7 +6601,7 @@
         <v>185</v>
       </c>
       <c r="B186" s="20" t="s">
-        <v>583</v>
+        <v>310</v>
       </c>
       <c r="C186" s="8" t="s">
         <v>98</v>
@@ -7447,7 +6627,7 @@
         <v>186</v>
       </c>
       <c r="B187" s="20" t="s">
-        <v>584</v>
+        <v>311</v>
       </c>
       <c r="C187" s="5" t="s">
         <v>98</v>
@@ -7473,7 +6653,7 @@
         <v>187</v>
       </c>
       <c r="B188" s="20" t="s">
-        <v>585</v>
+        <v>312</v>
       </c>
       <c r="C188" s="8" t="s">
         <v>98</v>
@@ -7499,7 +6679,7 @@
         <v>188</v>
       </c>
       <c r="B189" s="20" t="s">
-        <v>586</v>
+        <v>313</v>
       </c>
       <c r="C189" s="5" t="s">
         <v>98</v>
@@ -7525,7 +6705,7 @@
         <v>189</v>
       </c>
       <c r="B190" s="20" t="s">
-        <v>587</v>
+        <v>314</v>
       </c>
       <c r="C190" s="8" t="s">
         <v>98</v>
@@ -7551,7 +6731,7 @@
         <v>190</v>
       </c>
       <c r="B191" s="20" t="s">
-        <v>588</v>
+        <v>315</v>
       </c>
       <c r="C191" s="8" t="s">
         <v>98</v>
@@ -7577,7 +6757,7 @@
         <v>191</v>
       </c>
       <c r="B192" s="20" t="s">
-        <v>589</v>
+        <v>316</v>
       </c>
       <c r="C192" s="5" t="s">
         <v>98</v>
@@ -7603,7 +6783,7 @@
         <v>192</v>
       </c>
       <c r="B193" s="20" t="s">
-        <v>590</v>
+        <v>317</v>
       </c>
       <c r="C193" s="8" t="s">
         <v>98</v>
@@ -7629,7 +6809,7 @@
         <v>193</v>
       </c>
       <c r="B194" s="20" t="s">
-        <v>591</v>
+        <v>318</v>
       </c>
       <c r="C194" s="5" t="s">
         <v>98</v>
@@ -7655,7 +6835,7 @@
         <v>194</v>
       </c>
       <c r="B195" s="20" t="s">
-        <v>592</v>
+        <v>319</v>
       </c>
       <c r="C195" s="8" t="s">
         <v>98</v>
@@ -7681,7 +6861,7 @@
         <v>195</v>
       </c>
       <c r="B196" s="20" t="s">
-        <v>593</v>
+        <v>320</v>
       </c>
       <c r="C196" s="5" t="s">
         <v>98</v>
@@ -7707,7 +6887,7 @@
         <v>196</v>
       </c>
       <c r="B197" s="20" t="s">
-        <v>594</v>
+        <v>321</v>
       </c>
       <c r="C197" s="5" t="s">
         <v>98</v>
@@ -7733,7 +6913,7 @@
         <v>197</v>
       </c>
       <c r="B198" s="20" t="s">
-        <v>595</v>
+        <v>322</v>
       </c>
       <c r="C198" s="5" t="s">
         <v>98</v>
@@ -7759,7 +6939,7 @@
         <v>198</v>
       </c>
       <c r="B199" s="20" t="s">
-        <v>596</v>
+        <v>323</v>
       </c>
       <c r="C199" s="5" t="s">
         <v>98</v>
@@ -7785,7 +6965,7 @@
         <v>199</v>
       </c>
       <c r="B200" s="20" t="s">
-        <v>597</v>
+        <v>324</v>
       </c>
       <c r="C200" s="8" t="s">
         <v>98</v>
@@ -7811,7 +6991,7 @@
         <v>200</v>
       </c>
       <c r="B201" s="20" t="s">
-        <v>598</v>
+        <v>325</v>
       </c>
       <c r="C201" s="8" t="s">
         <v>98</v>
@@ -7837,7 +7017,7 @@
         <v>201</v>
       </c>
       <c r="B202" s="20" t="s">
-        <v>599</v>
+        <v>326</v>
       </c>
       <c r="C202" s="5" t="s">
         <v>98</v>
@@ -7863,7 +7043,7 @@
         <v>202</v>
       </c>
       <c r="B203" s="20" t="s">
-        <v>600</v>
+        <v>327</v>
       </c>
       <c r="C203" s="8" t="s">
         <v>98</v>
@@ -7889,7 +7069,7 @@
         <v>203</v>
       </c>
       <c r="B204" s="20" t="s">
-        <v>601</v>
+        <v>328</v>
       </c>
       <c r="C204" s="5" t="s">
         <v>98</v>
@@ -7915,7 +7095,7 @@
         <v>204</v>
       </c>
       <c r="B205" s="20" t="s">
-        <v>602</v>
+        <v>329</v>
       </c>
       <c r="C205" s="8" t="s">
         <v>98</v>
@@ -7941,7 +7121,7 @@
         <v>205</v>
       </c>
       <c r="B206" s="20" t="s">
-        <v>603</v>
+        <v>330</v>
       </c>
       <c r="C206" s="5" t="s">
         <v>98</v>
@@ -7967,7 +7147,7 @@
         <v>206</v>
       </c>
       <c r="B207" s="20" t="s">
-        <v>604</v>
+        <v>331</v>
       </c>
       <c r="C207" s="8" t="s">
         <v>98</v>
@@ -7993,7 +7173,7 @@
         <v>207</v>
       </c>
       <c r="B208" s="20" t="s">
-        <v>605</v>
+        <v>332</v>
       </c>
       <c r="C208" s="5" t="s">
         <v>98</v>
@@ -8019,7 +7199,7 @@
         <v>208</v>
       </c>
       <c r="B209" s="20" t="s">
-        <v>606</v>
+        <v>333</v>
       </c>
       <c r="C209" s="8" t="s">
         <v>98</v>
@@ -8045,7 +7225,7 @@
         <v>209</v>
       </c>
       <c r="B210" s="20" t="s">
-        <v>607</v>
+        <v>334</v>
       </c>
       <c r="C210" s="8" t="s">
         <v>98</v>
@@ -8071,7 +7251,7 @@
         <v>210</v>
       </c>
       <c r="B211" s="20" t="s">
-        <v>608</v>
+        <v>335</v>
       </c>
       <c r="C211" s="5" t="s">
         <v>98</v>
@@ -8097,7 +7277,7 @@
         <v>211</v>
       </c>
       <c r="B212" s="20" t="s">
-        <v>609</v>
+        <v>336</v>
       </c>
       <c r="C212" s="8" t="s">
         <v>98</v>
@@ -8123,7 +7303,7 @@
         <v>212</v>
       </c>
       <c r="B213" s="20" t="s">
-        <v>610</v>
+        <v>337</v>
       </c>
       <c r="C213" s="5" t="s">
         <v>98</v>
@@ -8149,7 +7329,7 @@
         <v>213</v>
       </c>
       <c r="B214" s="20" t="s">
-        <v>611</v>
+        <v>338</v>
       </c>
       <c r="C214" s="8" t="s">
         <v>98</v>
@@ -8175,7 +7355,7 @@
         <v>214</v>
       </c>
       <c r="B215" s="20" t="s">
-        <v>612</v>
+        <v>339</v>
       </c>
       <c r="C215" s="5" t="s">
         <v>98</v>
@@ -8201,7 +7381,7 @@
         <v>215</v>
       </c>
       <c r="B216" s="20" t="s">
-        <v>613</v>
+        <v>340</v>
       </c>
       <c r="C216" s="8" t="s">
         <v>98</v>
@@ -8227,7 +7407,7 @@
         <v>216</v>
       </c>
       <c r="B217" s="20" t="s">
-        <v>614</v>
+        <v>341</v>
       </c>
       <c r="C217" s="5" t="s">
         <v>98</v>
@@ -8253,7 +7433,7 @@
         <v>217</v>
       </c>
       <c r="B218" s="20" t="s">
-        <v>615</v>
+        <v>342</v>
       </c>
       <c r="C218" s="5" t="s">
         <v>98</v>
@@ -8279,7 +7459,7 @@
         <v>218</v>
       </c>
       <c r="B219" s="20" t="s">
-        <v>616</v>
+        <v>343</v>
       </c>
       <c r="C219" s="8" t="s">
         <v>98</v>
@@ -8305,7 +7485,7 @@
         <v>219</v>
       </c>
       <c r="B220" s="20" t="s">
-        <v>617</v>
+        <v>344</v>
       </c>
       <c r="C220" s="5" t="s">
         <v>98</v>
@@ -8331,7 +7511,7 @@
         <v>220</v>
       </c>
       <c r="B221" s="20" t="s">
-        <v>618</v>
+        <v>345</v>
       </c>
       <c r="C221" s="5" t="s">
         <v>98</v>
@@ -8357,7 +7537,7 @@
         <v>221</v>
       </c>
       <c r="B222" s="20" t="s">
-        <v>619</v>
+        <v>346</v>
       </c>
       <c r="C222" s="5" t="s">
         <v>98</v>
@@ -8383,7 +7563,7 @@
         <v>222</v>
       </c>
       <c r="B223" s="20" t="s">
-        <v>620</v>
+        <v>347</v>
       </c>
       <c r="C223" s="8" t="s">
         <v>98</v>
@@ -8409,7 +7589,7 @@
         <v>223</v>
       </c>
       <c r="B224" s="20" t="s">
-        <v>621</v>
+        <v>348</v>
       </c>
       <c r="C224" s="5" t="s">
         <v>98</v>
@@ -8435,7 +7615,7 @@
         <v>224</v>
       </c>
       <c r="B225" s="20" t="s">
-        <v>622</v>
+        <v>349</v>
       </c>
       <c r="C225" s="8" t="s">
         <v>98</v>
@@ -8461,7 +7641,7 @@
         <v>225</v>
       </c>
       <c r="B226" s="20" t="s">
-        <v>623</v>
+        <v>350</v>
       </c>
       <c r="C226" s="8" t="s">
         <v>98</v>
@@ -8487,7 +7667,7 @@
         <v>226</v>
       </c>
       <c r="B227" s="20" t="s">
-        <v>624</v>
+        <v>351</v>
       </c>
       <c r="C227" s="5" t="s">
         <v>98</v>
@@ -8513,7 +7693,7 @@
         <v>227</v>
       </c>
       <c r="B228" s="20" t="s">
-        <v>625</v>
+        <v>352</v>
       </c>
       <c r="C228" s="5" t="s">
         <v>98</v>
@@ -8539,7 +7719,7 @@
         <v>228</v>
       </c>
       <c r="B229" s="20" t="s">
-        <v>626</v>
+        <v>353</v>
       </c>
       <c r="C229" s="8" t="s">
         <v>98</v>
@@ -8565,7 +7745,7 @@
         <v>229</v>
       </c>
       <c r="B230" s="20" t="s">
-        <v>627</v>
+        <v>354</v>
       </c>
       <c r="C230" s="8" t="s">
         <v>98</v>
@@ -8591,7 +7771,7 @@
         <v>230</v>
       </c>
       <c r="B231" s="20" t="s">
-        <v>628</v>
+        <v>355</v>
       </c>
       <c r="C231" s="5" t="s">
         <v>98</v>
@@ -8617,7 +7797,7 @@
         <v>231</v>
       </c>
       <c r="B232" s="20" t="s">
-        <v>629</v>
+        <v>356</v>
       </c>
       <c r="C232" s="5" t="s">
         <v>98</v>
@@ -8643,7 +7823,7 @@
         <v>232</v>
       </c>
       <c r="B233" s="20" t="s">
-        <v>630</v>
+        <v>357</v>
       </c>
       <c r="C233" s="8" t="s">
         <v>98</v>
@@ -8669,7 +7849,7 @@
         <v>233</v>
       </c>
       <c r="B234" s="20" t="s">
-        <v>631</v>
+        <v>358</v>
       </c>
       <c r="C234" s="5" t="s">
         <v>98</v>
@@ -8695,7 +7875,7 @@
         <v>234</v>
       </c>
       <c r="B235" s="20" t="s">
-        <v>632</v>
+        <v>359</v>
       </c>
       <c r="C235" s="8" t="s">
         <v>98</v>
@@ -8721,7 +7901,7 @@
         <v>235</v>
       </c>
       <c r="B236" s="20" t="s">
-        <v>633</v>
+        <v>360</v>
       </c>
       <c r="C236" s="8" t="s">
         <v>98</v>
@@ -8747,7 +7927,7 @@
         <v>236</v>
       </c>
       <c r="B237" s="20" t="s">
-        <v>634</v>
+        <v>361</v>
       </c>
       <c r="C237" s="8" t="s">
         <v>98</v>
@@ -8773,7 +7953,7 @@
         <v>237</v>
       </c>
       <c r="B238" s="20" t="s">
-        <v>635</v>
+        <v>362</v>
       </c>
       <c r="C238" s="8" t="s">
         <v>98</v>
@@ -8799,7 +7979,7 @@
         <v>238</v>
       </c>
       <c r="B239" s="20" t="s">
-        <v>636</v>
+        <v>363</v>
       </c>
       <c r="C239" s="5" t="s">
         <v>98</v>
@@ -8825,7 +8005,7 @@
         <v>239</v>
       </c>
       <c r="B240" s="20" t="s">
-        <v>637</v>
+        <v>364</v>
       </c>
       <c r="C240" s="8" t="s">
         <v>98</v>
@@ -8851,7 +8031,7 @@
         <v>240</v>
       </c>
       <c r="B241" s="20" t="s">
-        <v>638</v>
+        <v>365</v>
       </c>
       <c r="C241" s="5" t="s">
         <v>98</v>
@@ -8877,7 +8057,7 @@
         <v>241</v>
       </c>
       <c r="B242" s="20" t="s">
-        <v>639</v>
+        <v>366</v>
       </c>
       <c r="C242" s="5" t="s">
         <v>98</v>
@@ -8903,7 +8083,7 @@
         <v>242</v>
       </c>
       <c r="B243" s="20" t="s">
-        <v>640</v>
+        <v>367</v>
       </c>
       <c r="C243" s="5" t="s">
         <v>98</v>
@@ -8929,7 +8109,7 @@
         <v>243</v>
       </c>
       <c r="B244" s="20" t="s">
-        <v>641</v>
+        <v>368</v>
       </c>
       <c r="C244" s="5" t="s">
         <v>98</v>
@@ -8955,7 +8135,7 @@
         <v>244</v>
       </c>
       <c r="B245" s="20" t="s">
-        <v>642</v>
+        <v>369</v>
       </c>
       <c r="C245" s="8" t="s">
         <v>98</v>
@@ -8981,7 +8161,7 @@
         <v>245</v>
       </c>
       <c r="B246" s="20" t="s">
-        <v>643</v>
+        <v>370</v>
       </c>
       <c r="C246" s="5" t="s">
         <v>98</v>
@@ -9007,7 +8187,7 @@
         <v>246</v>
       </c>
       <c r="B247" s="20" t="s">
-        <v>644</v>
+        <v>371</v>
       </c>
       <c r="C247" s="5" t="s">
         <v>98</v>
@@ -9033,7 +8213,7 @@
         <v>247</v>
       </c>
       <c r="B248" s="20" t="s">
-        <v>645</v>
+        <v>372</v>
       </c>
       <c r="C248" s="5" t="s">
         <v>98</v>
@@ -9059,7 +8239,7 @@
         <v>248</v>
       </c>
       <c r="B249" s="20" t="s">
-        <v>646</v>
+        <v>373</v>
       </c>
       <c r="C249" s="5" t="s">
         <v>98</v>
@@ -9085,7 +8265,7 @@
         <v>249</v>
       </c>
       <c r="B250" s="20" t="s">
-        <v>647</v>
+        <v>374</v>
       </c>
       <c r="C250" s="8" t="s">
         <v>98</v>
@@ -9111,7 +8291,7 @@
         <v>250</v>
       </c>
       <c r="B251" s="20" t="s">
-        <v>648</v>
+        <v>375</v>
       </c>
       <c r="C251" s="8" t="s">
         <v>98</v>
@@ -9137,7 +8317,7 @@
         <v>251</v>
       </c>
       <c r="B252" s="20" t="s">
-        <v>649</v>
+        <v>376</v>
       </c>
       <c r="C252" s="5" t="s">
         <v>98</v>
@@ -9163,7 +8343,7 @@
         <v>252</v>
       </c>
       <c r="B253" s="20" t="s">
-        <v>650</v>
+        <v>377</v>
       </c>
       <c r="C253" s="5" t="s">
         <v>98</v>
@@ -9189,7 +8369,7 @@
         <v>253</v>
       </c>
       <c r="B254" s="20" t="s">
-        <v>651</v>
+        <v>378</v>
       </c>
       <c r="C254" s="5" t="s">
         <v>98</v>
@@ -9215,7 +8395,7 @@
         <v>254</v>
       </c>
       <c r="B255" s="20" t="s">
-        <v>652</v>
+        <v>379</v>
       </c>
       <c r="C255" s="8" t="s">
         <v>98</v>
@@ -9241,7 +8421,7 @@
         <v>255</v>
       </c>
       <c r="B256" s="20" t="s">
-        <v>653</v>
+        <v>380</v>
       </c>
       <c r="C256" s="8" t="s">
         <v>98</v>
@@ -9267,7 +8447,7 @@
         <v>256</v>
       </c>
       <c r="B257" s="20" t="s">
-        <v>654</v>
+        <v>381</v>
       </c>
       <c r="C257" s="5" t="s">
         <v>98</v>
@@ -9293,7 +8473,7 @@
         <v>257</v>
       </c>
       <c r="B258" s="20" t="s">
-        <v>655</v>
+        <v>382</v>
       </c>
       <c r="C258" s="8" t="s">
         <v>98</v>
@@ -9319,7 +8499,7 @@
         <v>258</v>
       </c>
       <c r="B259" s="20" t="s">
-        <v>656</v>
+        <v>383</v>
       </c>
       <c r="C259" s="5" t="s">
         <v>98</v>
@@ -9345,7 +8525,7 @@
         <v>259</v>
       </c>
       <c r="B260" s="20" t="s">
-        <v>657</v>
+        <v>384</v>
       </c>
       <c r="C260" s="8" t="s">
         <v>98</v>
@@ -9371,7 +8551,7 @@
         <v>260</v>
       </c>
       <c r="B261" s="20" t="s">
-        <v>658</v>
+        <v>385</v>
       </c>
       <c r="C261" s="5" t="s">
         <v>98</v>
@@ -9397,7 +8577,7 @@
         <v>261</v>
       </c>
       <c r="B262" s="20" t="s">
-        <v>659</v>
+        <v>386</v>
       </c>
       <c r="C262" s="5" t="s">
         <v>98</v>
@@ -9423,7 +8603,7 @@
         <v>262</v>
       </c>
       <c r="B263" s="20" t="s">
-        <v>660</v>
+        <v>387</v>
       </c>
       <c r="C263" s="5" t="s">
         <v>98</v>
@@ -9449,7 +8629,7 @@
         <v>263</v>
       </c>
       <c r="B264" s="20" t="s">
-        <v>661</v>
+        <v>388</v>
       </c>
       <c r="C264" s="8" t="s">
         <v>98</v>
@@ -9475,7 +8655,7 @@
         <v>264</v>
       </c>
       <c r="B265" s="20" t="s">
-        <v>662</v>
+        <v>389</v>
       </c>
       <c r="C265" s="5" t="s">
         <v>98</v>
@@ -9501,7 +8681,7 @@
         <v>265</v>
       </c>
       <c r="B266" s="20" t="s">
-        <v>663</v>
+        <v>390</v>
       </c>
       <c r="C266" s="5" t="s">
         <v>98</v>
@@ -9527,7 +8707,7 @@
         <v>266</v>
       </c>
       <c r="B267" s="20" t="s">
-        <v>664</v>
+        <v>391</v>
       </c>
       <c r="C267" s="5" t="s">
         <v>98</v>
@@ -9553,7 +8733,7 @@
         <v>267</v>
       </c>
       <c r="B268" s="20" t="s">
-        <v>665</v>
+        <v>392</v>
       </c>
       <c r="C268" s="5" t="s">
         <v>98</v>
@@ -9579,7 +8759,7 @@
         <v>268</v>
       </c>
       <c r="B269" s="20" t="s">
-        <v>666</v>
+        <v>393</v>
       </c>
       <c r="C269" s="8" t="s">
         <v>98</v>
@@ -9605,7 +8785,7 @@
         <v>269</v>
       </c>
       <c r="B270" s="20" t="s">
-        <v>667</v>
+        <v>394</v>
       </c>
       <c r="C270" s="5" t="s">
         <v>98</v>
@@ -9631,7 +8811,7 @@
         <v>270</v>
       </c>
       <c r="B271" s="20" t="s">
-        <v>668</v>
+        <v>395</v>
       </c>
       <c r="C271" s="5" t="s">
         <v>98</v>
@@ -9657,7 +8837,7 @@
         <v>271</v>
       </c>
       <c r="B272" s="20" t="s">
-        <v>669</v>
+        <v>396</v>
       </c>
       <c r="C272" s="5" t="s">
         <v>98</v>
@@ -9683,7 +8863,7 @@
         <v>272</v>
       </c>
       <c r="B273" s="20" t="s">
-        <v>670</v>
+        <v>397</v>
       </c>
       <c r="C273" s="5" t="s">
         <v>98</v>
@@ -9709,7 +8889,7 @@
         <v>273</v>
       </c>
       <c r="B274" s="20" t="s">
-        <v>671</v>
+        <v>398</v>
       </c>
       <c r="C274" s="5" t="s">
         <v>98</v>
@@ -9741,16 +8921,16 @@
   <dimension ref="A1:J694"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.5"/>
-    <col min="2" max="2" customWidth="true" width="19.33203125"/>
-    <col min="3" max="3" customWidth="true" width="19.83203125"/>
-    <col min="4" max="4" customWidth="true" width="31.1640625"/>
-    <col min="5" max="5" customWidth="true" width="14.6640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="11.5"/>
-    <col min="7" max="7" customWidth="true" width="24.5"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="17.1640625"/>
-    <col min="9" max="9" customWidth="true" width="21.5"/>
-    <col min="10" max="10" customWidth="true" width="25.0"/>
+    <col min="1" max="1" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" customWidth="1"/>
+    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="4" max="4" width="31.1640625" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.5" customWidth="1"/>
+    <col min="8" max="8" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5" customWidth="1"/>
+    <col min="10" max="10" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="14" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>